<commit_message>
docs: generalize adecco evaluation scoring workbook
</commit_message>
<xml_diff>
--- a/outputs/browser_eval_result_mock_v2_logic/アデコ_ブラウザ評価_実行者モックv2_採点ロジック整理_2026-05-20.xlsx
+++ b/outputs/browser_eval_result_mock_v2_logic/アデコ_ブラウザ評価_実行者モックv2_採点ロジック整理_2026-05-20.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_全体整理" sheetId="1" r:id="Re09458a63ab04951"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_画面表示対応" sheetId="2" r:id="R62a4856f1e8e486e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_上部3項目" sheetId="3" r:id="Rf6e31650a4724d72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_6大カテゴリ採点基準" sheetId="4" r:id="Rac3fe43bbf0e4ebe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_6大カテゴリ一覧" sheetId="5" r:id="Rd7464209bd654abe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_12項目と改善インパクト" sheetId="6" r:id="Re2d16e2c57264af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_最優先改善領域ロジック" sheetId="7" r:id="R57e4d1fddeef403f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_会話フロー表記" sheetId="8" r:id="Re91d3f494e584d59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_総合点計算" sheetId="9" r:id="Rec5fe371aa73464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_次回アクション対応" sheetId="10" r:id="R842e1ab31fa84e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_全体整理" sheetId="1" r:id="R2862ea3686a74790"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_画面表示対応" sheetId="2" r:id="R5d819e7459ee48e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_上部3項目" sheetId="3" r:id="Ref6cfabe7e3a4581"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_6大カテゴリ採点基準" sheetId="4" r:id="Ra192908e3caf416c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_6大カテゴリ一覧" sheetId="5" r:id="R16ae796e1d424ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_12項目マスター" sheetId="6" r:id="Rbd2ed01609b0495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_最優先改善領域ロジック" sheetId="7" r:id="Rd02f215bb6a04499"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_会話フロー表記" sheetId="8" r:id="R11bb4d1690d9480b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_総合点計算" sheetId="9" r:id="Rf7a18cc8d91044a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_次回アクション対応" sheetId="10" r:id="Re23d6ed66d3e486e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -368,7 +368,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22.700000762939453" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="114.72000122070312" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="119.62999725341797" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -384,7 +384,7 @@
         <x:v>目的</x:v>
       </x:c>
       <x:c r="B2" s="17" t="str">
-        <x:v>実行者がロープレ後に見る採点結果モックv2と、その裏側の採点ロジックを1つに整理する。</x:v>
+        <x:v>ロープレ終了後のブラウザ採点結果画面と、その裏側の採点ロジックを汎用的に説明する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -392,7 +392,7 @@
         <x:v>画面方針</x:v>
       </x:c>
       <x:c r="B3" s="17" t="str">
-        <x:v>受講者向け画面では、総合点、3つの要約カード、6大カテゴリ、12項目の詳細、次回アクションを表示する。</x:v>
+        <x:v>実行者向け画面では、総合点、上部3項目、6大カテゴリ、必須ヒアリング12項目、会話フロー、次回アクションを整理して表示する。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -400,7 +400,7 @@
         <x:v>採点方針</x:v>
       </x:c>
       <x:c r="B4" s="17" t="str">
-        <x:v>AIが大カテゴリへ直接点を付けるのではなく、小カテゴリ/12項目を先に判定し、それを6大カテゴリへ集約する。</x:v>
+        <x:v>AIが大カテゴリへ直接点を付けるのではなく、小カテゴリや12項目を先に判定し、それを6大カテゴリへ集約する。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -408,31 +408,23 @@
         <x:v>最優先改善領域</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>必須ヒアリング12項目の中から、改善インパクトが最大の項目名をそのまま表示する。短縮名は使わない。</x:v>
+        <x:v>必須ヒアリング12項目の中から、改善インパクトが最大の項目名をそのまま表示する。AIが短縮名や別名を作らない。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
-        <x:v>今回モックの最優先改善領域</x:v>
+        <x:v>総合点</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
-        <x:v>連絡方法・スケジュール・ネクストステップ</x:v>
+        <x:v>6大カテゴリの点数合計で算出する。個別回の点数はこの資料には載せず、計算方法のみを定義する。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="16" t="str">
-        <x:v>総合点</x:v>
-      </x:c>
-      <x:c r="B7" s="17" t="str">
-        <x:v>6大カテゴリの点数合計。今回モックは 22.2 + 15.0 + 14.0 + 8.0 + 8.0 + 7.0 = 74.2点。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="18" t="str">
+      <x:c r="A7" s="18" t="str">
         <x:v>非言語評価</x:v>
       </x:c>
-      <x:c r="B8" s="19" t="str">
-        <x:v>商談時の振る舞いは、現時点では会話ログのみをもとに採点する。画面には米印で控えめに表示する。</x:v>
+      <x:c r="B7" s="19" t="str">
+        <x:v>商談時の振る舞いは、現時点では会話ログのみをもとに採点する。声量・表情・視線・姿勢などは直接評価対象にしない。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -445,16 +437,16 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="31.290000915527344" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="68.0999984741211" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="75.45999908447266" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="26" t="str">
-        <x:v>不足項目</x:v>
+        <x:v>不足領域</x:v>
       </x:c>
       <x:c r="B1" s="39" t="str">
-        <x:v>次回質問/行動例</x:v>
+        <x:v>次回質問/行動例の作り方</x:v>
       </x:c>
       <x:c r="C1" s="27" t="str">
         <x:v>画面上の出し方</x:v>
@@ -465,7 +457,7 @@
         <x:v>連絡方法・スケジュール・ネクストステップ</x:v>
       </x:c>
       <x:c r="B2" s="34" t="str">
-        <x:v>最後に、候補者像・提案期限・連絡方法・双方の次行動を一文で要約する。</x:v>
+        <x:v>候補者像・提案期限・連絡方法・双方の次行動を一文で要約する練習に落とす。</x:v>
       </x:c>
       <x:c r="C2" s="17" t="str">
         <x:v>次回トレーニングアクション</x:v>
@@ -476,21 +468,32 @@
         <x:v>競合・見学・決定プロセス</x:v>
       </x:c>
       <x:c r="B3" s="34" t="str">
-        <x:v>候補者を提案した後、職場見学から決定まではどなたが、何日くらいで判断されますか。</x:v>
+        <x:v>職場見学後の決定者、判断日数、競合状況、独占余地を確認する質問例にする。</x:v>
       </x:c>
       <x:c r="C3" s="17" t="str">
         <x:v>次回に効く要点/次回の質問例</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="18" t="str">
+      <x:c r="A4" s="16" t="str">
         <x:v>優先順位の明確化</x:v>
       </x:c>
-      <x:c r="B4" s="35" t="str">
-        <x:v>絶対条件、できれば条件、緩和できる条件に分けるとどうなりますか。</x:v>
-      </x:c>
-      <x:c r="C4" s="19" t="str">
+      <x:c r="B4" s="34" t="str">
+        <x:v>絶対条件、できれば条件、緩和できる条件に分ける質問例にする。</x:v>
+      </x:c>
+      <x:c r="C4" s="17" t="str">
         <x:v>改善ポイント/練習アクション</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="18" t="str">
+        <x:v>ヒアリングスキル</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="str">
+        <x:v>質問が抽象的だった箇所を、オープン質問からクローズ確認へつなぐ練習にする。</x:v>
+      </x:c>
+      <x:c r="C5" s="19" t="str">
+        <x:v>次回トレーニングアクション</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -517,7 +520,7 @@
         <x:v>表示項目</x:v>
       </x:c>
       <x:c r="C1" s="39" t="str">
-        <x:v>今回の表示</x:v>
+        <x:v>表示内容/形式</x:v>
       </x:c>
       <x:c r="D1" s="39" t="str">
         <x:v>意味</x:v>
@@ -534,7 +537,7 @@
         <x:v>総合評価</x:v>
       </x:c>
       <x:c r="C2" s="34" t="str">
-        <x:v>74.2 / 100, Grade B</x:v>
+        <x:v>総合点 / 100、Grade</x:v>
       </x:c>
       <x:c r="D2" s="34" t="str">
         <x:v>ロープレ全体の最終評価。</x:v>
@@ -551,13 +554,13 @@
         <x:v>評価信頼度</x:v>
       </x:c>
       <x:c r="C3" s="34" t="str">
-        <x:v>high</x:v>
+        <x:v>high / medium / low</x:v>
       </x:c>
       <x:c r="D3" s="34" t="str">
         <x:v>採点に使う会話ログが十分かどうか。</x:v>
       </x:c>
       <x:c r="E3" s="17" t="str">
-        <x:v>sales/client両方の発話、欠落、評価不能項目などをもとに判定。</x:v>
+        <x:v>営業側・顧客側の発話、欠落、評価不能項目などをもとに判定。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -568,10 +571,10 @@
         <x:v>ヒアリング達成度</x:v>
       </x:c>
       <x:c r="C4" s="34" t="str">
-        <x:v>74%</x:v>
+        <x:v>パーセンテージ</x:v>
       </x:c>
       <x:c r="D4" s="34" t="str">
-        <x:v>必須ヒアリングをどれくらい取れたか。</x:v>
+        <x:v>必須ヒアリングをどれくらい取得できたか。</x:v>
       </x:c>
       <x:c r="E4" s="17" t="str">
         <x:v>12項目の重み付き取得率。</x:v>
@@ -585,7 +588,7 @@
         <x:v>完全取得 / 部分取得 / 未取得</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>7 / 3 / 2</x:v>
+        <x:v>件数内訳</x:v>
       </x:c>
       <x:c r="D5" s="34" t="str">
         <x:v>12項目の判定内訳。</x:v>
@@ -602,13 +605,13 @@
         <x:v>最優先改善領域</x:v>
       </x:c>
       <x:c r="C6" s="34" t="str">
-        <x:v>連絡方法・スケジュール・ネクストステップ</x:v>
+        <x:v>12項目マスターの項目名</x:v>
       </x:c>
       <x:c r="D6" s="34" t="str">
         <x:v>最初に改善すると点数・実務効果が大きい項目。</x:v>
       </x:c>
       <x:c r="E6" s="17" t="str">
-        <x:v>改善インパクト = 重み × (1 - 取得率) が最大の12項目名をそのまま表示。</x:v>
+        <x:v>改善インパクト = 重み × (1 - 取得率) が最大の項目名をそのまま表示。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -619,7 +622,7 @@
         <x:v>6大カテゴリ</x:v>
       </x:c>
       <x:c r="C7" s="34" t="str">
-        <x:v>30/20/20/10/10/10</x:v>
+        <x:v>30/20/20/10/10/10点のカテゴリ別結果</x:v>
       </x:c>
       <x:c r="D7" s="34" t="str">
         <x:v>お客様要望の100点満点配点に沿った評価。</x:v>
@@ -673,10 +676,9 @@
   <x:cols>
     <x:col min="1" max="1" width="6.75" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="27.610000610351562" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="31.290000915527344" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="55.83000183105469" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="43.560001373291016" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="50.91999816894531" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="55.83000183105469" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="50.91999816894531" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -687,16 +689,13 @@
         <x:v>表示名</x:v>
       </x:c>
       <x:c r="C1" s="39" t="str">
-        <x:v>今回表示</x:v>
+        <x:v>意味</x:v>
       </x:c>
       <x:c r="D1" s="39" t="str">
-        <x:v>意味</x:v>
-      </x:c>
-      <x:c r="E1" s="39" t="str">
         <x:v>計算/選定方法</x:v>
       </x:c>
-      <x:c r="F1" s="27" t="str">
-        <x:v>なぜ上部に置くか</x:v>
+      <x:c r="E1" s="27" t="str">
+        <x:v>表示上の注意</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="24" hidden="0" customHeight="1">
@@ -707,16 +706,13 @@
         <x:v>ヒアリング達成度</x:v>
       </x:c>
       <x:c r="C2" s="34" t="str">
-        <x:v>74%</x:v>
+        <x:v>必須ヒアリング12項目を、重要度込みでどれくらい取得できたか。</x:v>
       </x:c>
       <x:c r="D2" s="34" t="str">
-        <x:v>必須ヒアリング12項目を、重要度込みでどれくらい取得できたか。</x:v>
-      </x:c>
-      <x:c r="E2" s="34" t="str">
         <x:v>12項目それぞれを 完全取得=1 / 部分取得=0.5 / 未取得=0 とし、重み付き取得率を計算する。</x:v>
       </x:c>
-      <x:c r="F2" s="17" t="str">
-        <x:v>実行者が最初に、必要情報をどれくらい取れたか把握できるため。</x:v>
+      <x:c r="E2" s="17" t="str">
+        <x:v>単純な項目数ではなく、重みを考慮した達成度として表示する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" hidden="0" customHeight="1">
@@ -727,19 +723,16 @@
         <x:v>完全取得 / 部分取得 / 未取得</x:v>
       </x:c>
       <x:c r="C3" s="34" t="str">
-        <x:v>7 / 3 / 2</x:v>
+        <x:v>12項目の判定内訳。何項目が十分で、何項目が浅く、何項目が未取得かを示す。</x:v>
       </x:c>
       <x:c r="D3" s="34" t="str">
-        <x:v>12項目の判定内訳。何項目が十分で、何項目が浅く、何項目が未取得かを示す。</x:v>
-      </x:c>
-      <x:c r="E3" s="34" t="str">
         <x:v>12項目の判定結果を件数集計する。</x:v>
       </x:c>
-      <x:c r="F3" s="17" t="str">
-        <x:v>ヒアリング達成度だけでは分からない、取得状況のばらつきを把握できるため。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="36" hidden="0" customHeight="1">
+      <x:c r="E3" s="17" t="str">
+        <x:v>ラベルは「取得」ではなく「完全取得」とし、判定の意味を明確にする。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" hidden="0" customHeight="1">
       <x:c r="A4" s="18" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -747,16 +740,13 @@
         <x:v>最優先改善領域</x:v>
       </x:c>
       <x:c r="C4" s="35" t="str">
-        <x:v>連絡方法・スケジュール・ネクストステップ</x:v>
+        <x:v>次回最初に改善すると点数・実務効果が大きい必須ヒアリング項目。</x:v>
       </x:c>
       <x:c r="D4" s="35" t="str">
-        <x:v>次回最初に改善すると点数・実務効果が大きい必須ヒアリング項目。</x:v>
-      </x:c>
-      <x:c r="E4" s="35" t="str">
-        <x:v>改善インパクト = 重み × (1 - 取得率)。最大の12項目名をそのまま表示する。AIが自由に短縮名を作らない。</x:v>
-      </x:c>
-      <x:c r="F4" s="19" t="str">
-        <x:v>次に何を直すべきか、詳細表を読まなくても一目で分かるため。</x:v>
+        <x:v>改善インパクト = 重み × (1 - 取得率)。最大の12項目名をそのまま表示する。</x:v>
+      </x:c>
+      <x:c r="E4" s="19" t="str">
+        <x:v>短縮名やAIが作った別名ではなく、12項目マスターの名称をそのまま使う。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -775,7 +765,7 @@
     <x:col min="5" max="5" width="50.91999816894531" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="63.189998626708984" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="53.369998931884766" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16.559999465942383" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="46.0099983215332" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -801,10 +791,10 @@
         <x:v>点数化の考え方</x:v>
       </x:c>
       <x:c r="H1" s="27" t="str">
-        <x:v>今回モック表示</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="48" hidden="0" customHeight="1">
+        <x:v>画面表示方針</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="144" hidden="0" customHeight="1">
       <x:c r="A2" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -818,19 +808,30 @@
         <x:v>お客様要望: 聞くべき項目をもれなく正確に聞けているか。Excel 05_採点_QA: 必須ヒアリング12項目。</x:v>
       </x:c>
       <x:c r="E2" s="34" t="str">
-        <x:v>AIがいきなり30点を直接採点すると揺れやすいため、Excel 05_採点_QA の12項目を先に判定する。</x:v>
+        <x:v>大カテゴリへ直接30点を付けると揺れやすいため、必須ヒアリング12項目を先に判定してから集約する。</x:v>
       </x:c>
       <x:c r="F2" s="34" t="str">
-        <x:v>募集背景、業務内容・1日の流れ、業務量・繁忙・引継ぎ、就業開始日・期間、曜日・時間・残業・リモート、料金・交通費・直接雇用、必須要件・ベター要件、優先順位の明確化、職場環境、雰囲気・NG人物像、競合・見学・決定プロセス、連絡方法・スケジュール・ネクストステップ。</x:v>
+        <x:v>・募集背景
+・業務内容・1日の流れ
+・業務量・繁忙・引継ぎ
+・就業開始日・期間
+・曜日・時間・残業・リモート
+・料金・交通費・直接雇用
+・必須要件・ベター要件
+・優先順位の明確化
+・職場環境
+・雰囲気・NG人物像
+・競合・見学・決定プロセス
+・連絡方法・スケジュール・ネクストステップ</x:v>
       </x:c>
       <x:c r="G2" s="34" t="str">
-        <x:v>12項目を 完全取得=1 / 部分取得=0.5 / 未取得=0 で判定し、重み付き取得率を算出。その取得率を30点満点に換算する。</x:v>
+        <x:v>12項目を 完全取得=1 / 部分取得=0.5 / 未取得=0 で判定し、重み付き取得率を算出する。その取得率を30点満点に換算する。</x:v>
       </x:c>
       <x:c r="H2" s="17" t="str">
-        <x:v>22.2 / 30</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="36" hidden="0" customHeight="1">
+        <x:v>6大カテゴリ欄には30点満点の結果を表示し、詳細欄には12項目の判定内訳を表示する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="60" hidden="0" customHeight="1">
       <x:c r="A3" s="16" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -844,19 +845,23 @@
         <x:v>お客様要望: 質問内容の明確さ、オープン/クローズ、第三者話法、構造化と要約。Excel 03_ヒアリング設計: 例の質問、次の深掘り、なぜ効くか。</x:v>
       </x:c>
       <x:c r="E3" s="34" t="str">
-        <x:v>質問項目を聞いたかだけでなく、相手が答えやすい聞き方・深掘り・要約ができたかを評価するため。</x:v>
+        <x:v>項目を聞いたかだけでなく、相手が答えやすい聞き方・深掘り・要約ができたかを評価するため。</x:v>
       </x:c>
       <x:c r="F3" s="34" t="str">
-        <x:v>質問が明確だったか、オープン質問とクローズ質問を使い分けたか、第三者話法を使えたか、相手の回答を受けて深掘りできたか、要約して認識合わせできたか。</x:v>
+        <x:v>・質問が明確だったか
+・オープン質問とクローズ質問を使い分けたか
+・第三者話法を使えたか
+・相手の回答を受けて深掘りできたか
+・要約して認識合わせできたか</x:v>
       </x:c>
       <x:c r="G3" s="34" t="str">
-        <x:v>各小カテゴリを0〜4で判定し、平均または重み付き平均を20点満点に換算する。</x:v>
+        <x:v>各小カテゴリを段階評価し、平均または重み付き平均を20点満点に換算する。</x:v>
       </x:c>
       <x:c r="H3" s="17" t="str">
-        <x:v>15.0 / 20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="48" hidden="0" customHeight="1">
+        <x:v>6大カテゴリ欄には20点満点の結果を表示し、コメントでは良かった聞き方と改善すべき聞き方を分けて示す。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="60" hidden="0" customHeight="1">
       <x:c r="A4" s="16" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -873,16 +878,20 @@
         <x:v>人選担当が候補者を選びやすいように、条件の優先順位を整理できたかを見るため。</x:v>
       </x:c>
       <x:c r="F4" s="34" t="str">
-        <x:v>絶対条件を聞けたか、ベター条件を聞けたか、緩和できる条件を聞けたか、経験・スキル・開始日・人柄の優先順位を聞けたか、人選担当が候補者を選びやすい形に整理できたか。</x:v>
+        <x:v>・絶対条件を聞けたか
+・ベター条件を聞けたか
+・緩和できる条件を聞けたか
+・経験・スキル・開始日・人柄の優先順位を聞けたか
+・候補者選定に使える形へ整理できたか</x:v>
       </x:c>
       <x:c r="G4" s="34" t="str">
-        <x:v>優先順位に関する小カテゴリを0〜4で判定し、20点満点に換算する。年齢・性別など不適切要件は、そのまま深掘りした場合は加点せず、職務関連要件に言い換えた場合のみ評価する。</x:v>
+        <x:v>優先順位に関する小カテゴリを段階評価し、20点満点に換算する。年齢・性別など不適切要件は、職務関連要件に言い換えて確認できた場合のみ評価する。</x:v>
       </x:c>
       <x:c r="H4" s="17" t="str">
-        <x:v>14.0 / 20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="48" hidden="0" customHeight="1">
+        <x:v>6大カテゴリ欄には20点満点の結果を表示し、不足が大きい場合は次回質問例に優先順位整理の質問を出す。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="84" hidden="0" customHeight="1">
       <x:c r="A5" s="16" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -899,16 +908,22 @@
         <x:v>話があちこちに飛ばず、初回商談として自然な順番で進行できたかを見るため。</x:v>
       </x:c>
       <x:c r="F5" s="34" t="str">
-        <x:v>導入、背景、業務分解、優先順位、職場環境、競合・決定、要約・終話。</x:v>
+        <x:v>・導入
+・背景
+・業務分解
+・優先順位
+・職場環境
+・競合・決定
+・要約・終話</x:v>
       </x:c>
       <x:c r="G5" s="34" t="str">
-        <x:v>会話フロー各ステージを 実施/部分/不足 で判定し、流れの自然さを0〜4で評価して10点満点に換算する。</x:v>
+        <x:v>会話フロー各ステージを 実施 / 部分 / 不足 で判定し、流れの自然さを10点満点に換算する。</x:v>
       </x:c>
       <x:c r="H5" s="17" t="str">
-        <x:v>8.0 / 10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="36" hidden="0" customHeight="1">
+        <x:v>6大カテゴリ欄には10点満点の結果を表示し、会話フロー欄には各ステージの進み具合を表示する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="60" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -922,19 +937,23 @@
         <x:v>お客様要望: 声の大きさ、活力、まどろっこしくないか、傾聴姿勢、表情、視線、姿勢、メモ中の態度。</x:v>
       </x:c>
       <x:c r="E6" s="34" t="str">
-        <x:v>振る舞いは重要だが、今回のブラウザ評価は会話ログが根拠のため、評価可能範囲を分けて扱う必要がある。</x:v>
+        <x:v>振る舞いは重要だが、ブラウザ評価は会話ログが根拠のため、評価可能範囲を明確に分ける必要がある。</x:v>
       </x:c>
       <x:c r="F6" s="34" t="str">
-        <x:v>発話が簡潔か、相手の回答を受けて応答できているか、傾聴姿勢が会話上伝わるか、一方的な説明や詰問になっていないか。</x:v>
+        <x:v>・発話が簡潔か
+・相手の回答を受けて応答できているか
+・傾聴姿勢が会話上伝わるか
+・一方的な説明になっていないか
+・詰問調になっていないか</x:v>
       </x:c>
       <x:c r="G6" s="34" t="str">
-        <x:v>会話ログで評価可能な小カテゴリだけを0〜4で判定し、10点満点に換算する。声量・表情・視線・姿勢・メモ中の態度は現時点では直接評価しない。</x:v>
+        <x:v>会話ログで評価可能な小カテゴリだけを段階評価し、10点満点に換算する。声量・表情・視線・姿勢・メモ中の態度は直接評価しない。</x:v>
       </x:c>
       <x:c r="H6" s="17" t="str">
-        <x:v>8.0 / 10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="48" hidden="0" customHeight="1">
+        <x:v>6大カテゴリ欄には10点満点の結果を表示し、画面上には「会話ログのみをもとに採点」と米印で控えめに記載する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="60" hidden="0" customHeight="1">
       <x:c r="A7" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -945,19 +964,23 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D7" s="35" t="str">
-        <x:v>お客様要望: 今後のスケジュールとネクストアクションを具体的な期日と行動ベースで合意できているか。Excel 05_採点_QA: 連絡方法・スケジュール・ネクストステップが14点で最重。</x:v>
+        <x:v>お客様要望: 今後のスケジュールとネクストアクションを具体的な期日と行動ベースで合意できているか。Excel 05_採点_QA: 連絡方法・スケジュール・ネクストステップ。</x:v>
       </x:c>
       <x:c r="E7" s="35" t="str">
         <x:v>終盤の合意形成は、初回商談が次の実行に進むかを左右するため。</x:v>
       </x:c>
       <x:c r="F7" s="35" t="str">
-        <x:v>担当者への連絡方法を確認したか、候補者提示日を合意したか、職場見学の進め方を確認したか、決定者と決定までの日数を確認したか、双方の次行動を期日付きで合意したか。</x:v>
+        <x:v>・担当者への連絡方法を確認したか
+・候補者提示日を合意したか
+・職場見学の進め方を確認したか
+・決定者と決定までの日数を確認したか
+・双方の次行動を期日付きで合意したか</x:v>
       </x:c>
       <x:c r="G7" s="35" t="str">
-        <x:v>クロージング小カテゴリを0〜4で判定し、10点満点に換算する。12項目側では「連絡方法・スケジュール・ネクストステップ」の不足も強く反映される。</x:v>
+        <x:v>クロージング小カテゴリを段階評価し、10点満点に換算する。12項目側では「連絡方法・スケジュール・ネクストステップ」の不足も強く反映する。</x:v>
       </x:c>
       <x:c r="H7" s="19" t="str">
-        <x:v>7.0 / 10</x:v>
+        <x:v>6大カテゴリ欄には10点満点の結果を表示し、不足があれば次回アクションに期日・行動ベースの合意を出す。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -973,7 +996,7 @@
     <x:col min="2" max="2" width="7.980000019073486" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="52.150001525878906" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="54.599998474121094" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17.790000915527344" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="43.560001373291016" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -993,7 +1016,7 @@
         <x:v>画面表示</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="24" hidden="0" customHeight="1">
+    <x:row r="2" ht="36" hidden="0" customHeight="1">
       <x:c r="A2" s="16" t="str">
         <x:v>ヒアリング項目の網羅性</x:v>
       </x:c>
@@ -1001,16 +1024,18 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="C2" s="34" t="str">
-        <x:v>必須ヒアリング12項目の取得状況、順番の合理性、候補者提案に使える粒度</x:v>
+        <x:v>・必須ヒアリング12項目の取得状況
+・聞く順番の合理性
+・候補者提案に使える粒度</x:v>
       </x:c>
       <x:c r="D2" s="34" t="str">
-        <x:v>12項目の重み付き取得率 × 30点。今回例: 74% × 30 = 22.2点。</x:v>
+        <x:v>12項目の重み付き取得率を30点満点に換算する。</x:v>
       </x:c>
       <x:c r="E2" s="17" t="str">
-        <x:v>22.2 / 30</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="24" hidden="0" customHeight="1">
+        <x:v>カテゴリ別スコアと、12項目詳細を併記する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="72" hidden="0" customHeight="1">
       <x:c r="A3" s="16" t="str">
         <x:v>ヒアリングスキル</x:v>
       </x:c>
@@ -1018,16 +1043,21 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C3" s="34" t="str">
-        <x:v>質問の明確さ、オープン/クローズ、第三者話法、構造化、要約、相手回答を受けた深掘り</x:v>
+        <x:v>・質問の明確さ
+・オープン/クローズの使い分け
+・第三者話法
+・構造化
+・要約
+・相手回答を受けた深掘り</x:v>
       </x:c>
       <x:c r="D3" s="34" t="str">
-        <x:v>各小カテゴリを0〜4で判定し、平均を20点換算。</x:v>
+        <x:v>各小カテゴリを段階評価し、20点満点に換算する。</x:v>
       </x:c>
       <x:c r="E3" s="17" t="str">
-        <x:v>15.0 / 20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="24" hidden="0" customHeight="1">
+        <x:v>カテゴリ別スコアと、良かった聞き方/改善すべき聞き方を表示する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="48" hidden="0" customHeight="1">
       <x:c r="A4" s="16" t="str">
         <x:v>優先順位の明確化</x:v>
       </x:c>
@@ -1035,16 +1065,19 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="C4" s="34" t="str">
-        <x:v>必須条件、歓迎条件、緩和可能条件、経験/スキル/開始日/人柄の優先順位</x:v>
+        <x:v>・必須条件
+・歓迎条件
+・緩和可能条件
+・経験/スキル/開始日/人柄の優先順位</x:v>
       </x:c>
       <x:c r="D4" s="34" t="str">
-        <x:v>小カテゴリを0〜4で判定し、平均または重要小カテゴリを加重して20点換算。</x:v>
+        <x:v>小カテゴリを段階評価し、20点満点に換算する。</x:v>
       </x:c>
       <x:c r="E4" s="17" t="str">
-        <x:v>14.0 / 20</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="24" hidden="0" customHeight="1">
+        <x:v>カテゴリ別スコアと、優先順位整理の不足を表示する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="108" hidden="0" customHeight="1">
       <x:c r="A5" s="16" t="str">
         <x:v>商談の全体構成力</x:v>
       </x:c>
@@ -1052,16 +1085,24 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>導入、背景、業務分解、条件整理、優先順位、職場環境、競合/決定、要約、終話</x:v>
+        <x:v>・導入
+・背景
+・業務分解
+・条件整理
+・優先順位
+・職場環境
+・競合/決定
+・要約
+・終話</x:v>
       </x:c>
       <x:c r="D5" s="34" t="str">
-        <x:v>会話フロー達成度を0〜4で判定し10点換算。</x:v>
+        <x:v>会話フロー達成度を10点満点に換算する。</x:v>
       </x:c>
       <x:c r="E5" s="17" t="str">
-        <x:v>8.0 / 10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+        <x:v>カテゴリ別スコアと、会話フロー表を表示する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="60" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
         <x:v>商談時の振る舞い</x:v>
       </x:c>
@@ -1069,16 +1110,20 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C6" s="34" t="str">
-        <x:v>簡潔さ、応答、傾聴、活力ある言い回し、一方的説明や詰問の有無</x:v>
+        <x:v>・簡潔さ
+・応答
+・傾聴
+・活力ある言い回し
+・一方的説明や詰問の有無</x:v>
       </x:c>
       <x:c r="D6" s="34" t="str">
-        <x:v>会話ログで評価可能な小カテゴリだけを0〜4で判定し10点換算。</x:v>
+        <x:v>会話ログで評価可能な小カテゴリだけを10点満点に換算する。</x:v>
       </x:c>
       <x:c r="E6" s="17" t="str">
-        <x:v>8.0 / 10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="24" hidden="0" customHeight="1">
+        <x:v>カテゴリ別スコアと、会話ログのみを根拠にする注意書きを表示する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="72" hidden="0" customHeight="1">
       <x:c r="A7" s="18" t="str">
         <x:v>クロージング</x:v>
       </x:c>
@@ -1086,13 +1131,18 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="C7" s="35" t="str">
-        <x:v>連絡方法、候補提示日、職場見学、決定プロセス、双方の次行動、期日合意</x:v>
+        <x:v>・連絡方法
+・候補提示日
+・職場見学
+・決定プロセス
+・双方の次行動
+・期日合意</x:v>
       </x:c>
       <x:c r="D7" s="35" t="str">
-        <x:v>クロージング小カテゴリを0〜4で判定し10点換算。</x:v>
+        <x:v>クロージング小カテゴリを10点満点に換算する。</x:v>
       </x:c>
       <x:c r="E7" s="19" t="str">
-        <x:v>7.0 / 10</x:v>
+        <x:v>カテゴリ別スコアと、次回アクションの不足を表示する。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1107,11 +1157,9 @@
     <x:col min="1" max="1" width="5.519999980926514" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="34.970001220703125" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="7.980000019073486" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11.65999984741211" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="7.980000019073486" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="50.91999816894531" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="25.149999618530273" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22.700000762939453" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="68.0999984741211" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="26.3799991607666" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -1125,18 +1173,12 @@
         <x:v>重み</x:v>
       </x:c>
       <x:c r="D1" s="39" t="str">
-        <x:v>今回判定</x:v>
+        <x:v>判定単位</x:v>
       </x:c>
       <x:c r="E1" s="39" t="str">
-        <x:v>取得率</x:v>
-      </x:c>
-      <x:c r="F1" s="39" t="str">
-        <x:v>改善インパクト</x:v>
-      </x:c>
-      <x:c r="G1" s="39" t="str">
-        <x:v>根拠・不足</x:v>
-      </x:c>
-      <x:c r="H1" s="27" t="str">
+        <x:v>判定観点</x:v>
+      </x:c>
+      <x:c r="F1" s="27" t="str">
         <x:v>主に影響する大カテゴリ</x:v>
       </x:c>
     </x:row>
@@ -1151,18 +1193,12 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="D2" s="34" t="str">
-        <x:v>完全取得</x:v>
-      </x:c>
-      <x:c r="E2" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" s="34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G2" s="34" t="str">
-        <x:v>増員背景と現行ベンダーへの不満を確認。</x:v>
-      </x:c>
-      <x:c r="H2" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E2" s="34" t="str">
+        <x:v>募集背景、増員/交代、その理由を確認できているか。</x:v>
+      </x:c>
+      <x:c r="F2" s="17" t="str">
         <x:v>網羅性</x:v>
       </x:c>
     </x:row>
@@ -1177,18 +1213,12 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="D3" s="34" t="str">
-        <x:v>完全取得</x:v>
-      </x:c>
-      <x:c r="E3" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F3" s="34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G3" s="34" t="str">
-        <x:v>受発注、納期調整、メール対応まで確認。</x:v>
-      </x:c>
-      <x:c r="H3" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E3" s="34" t="str">
+        <x:v>職種・業務の大枠、業務内容、1日の流れを確認できているか。</x:v>
+      </x:c>
+      <x:c r="F3" s="17" t="str">
         <x:v>網羅性</x:v>
       </x:c>
     </x:row>
@@ -1203,18 +1233,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D4" s="34" t="str">
-        <x:v>部分取得</x:v>
-      </x:c>
-      <x:c r="E4" s="34" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="F4" s="34" t="n">
-        <x:v>3.5</x:v>
-      </x:c>
-      <x:c r="G4" s="34" t="str">
-        <x:v>繁忙サイクルは確認。件数感と独り立ち時期が浅い。</x:v>
-      </x:c>
-      <x:c r="H4" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E4" s="34" t="str">
+        <x:v>業務量、繁忙サイクル、引継ぎ方法・期間を確認できているか。</x:v>
+      </x:c>
+      <x:c r="F4" s="17" t="str">
         <x:v>網羅性</x:v>
       </x:c>
     </x:row>
@@ -1229,18 +1253,12 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D5" s="34" t="str">
-        <x:v>完全取得</x:v>
-      </x:c>
-      <x:c r="E5" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F5" s="34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G5" s="34" t="str">
-        <x:v>開始希望と契約期間を確認。</x:v>
-      </x:c>
-      <x:c r="H5" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E5" s="34" t="str">
+        <x:v>開始日、契約期間、更新見込みを確認できているか。</x:v>
+      </x:c>
+      <x:c r="F5" s="17" t="str">
         <x:v>網羅性</x:v>
       </x:c>
     </x:row>
@@ -1255,18 +1273,12 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="D6" s="34" t="str">
-        <x:v>完全取得</x:v>
-      </x:c>
-      <x:c r="E6" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F6" s="34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G6" s="34" t="str">
-        <x:v>候補者説明に使える粒度で確認。</x:v>
-      </x:c>
-      <x:c r="H6" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E6" s="34" t="str">
+        <x:v>曜日、時間、休憩、残業、リモート有無・頻度を確認できているか。</x:v>
+      </x:c>
+      <x:c r="F6" s="17" t="str">
         <x:v>網羅性</x:v>
       </x:c>
     </x:row>
@@ -1281,18 +1293,12 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D7" s="34" t="str">
-        <x:v>部分取得</x:v>
-      </x:c>
-      <x:c r="E7" s="34" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="F7" s="34" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G7" s="34" t="str">
-        <x:v>請求金額は確認。直接雇用可能性が未確認。</x:v>
-      </x:c>
-      <x:c r="H7" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E7" s="34" t="str">
+        <x:v>請求金額、交通費、直接雇用可能性を確認できているか。</x:v>
+      </x:c>
+      <x:c r="F7" s="17" t="str">
         <x:v>網羅性</x:v>
       </x:c>
     </x:row>
@@ -1307,18 +1313,12 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D8" s="34" t="str">
-        <x:v>完全取得</x:v>
-      </x:c>
-      <x:c r="E8" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F8" s="34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G8" s="34" t="str">
-        <x:v>受発注経験、OA、基幹システム経験を確認。</x:v>
-      </x:c>
-      <x:c r="H8" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E8" s="34" t="str">
+        <x:v>最低条件、ベター条件、必要資格・OAスキルを確認できているか。</x:v>
+      </x:c>
+      <x:c r="F8" s="17" t="str">
         <x:v>網羅性/優先順位</x:v>
       </x:c>
     </x:row>
@@ -1333,18 +1333,12 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D9" s="34" t="str">
-        <x:v>部分取得</x:v>
-      </x:c>
-      <x:c r="E9" s="34" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="F9" s="34" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G9" s="34" t="str">
-        <x:v>必須条件・歓迎条件・緩和可能条件の切り分けが一段不足。</x:v>
-      </x:c>
-      <x:c r="H9" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E9" s="34" t="str">
+        <x:v>must/want、緩和可能条件、候補者選定上の優先順位を確認できているか。</x:v>
+      </x:c>
+      <x:c r="F9" s="17" t="str">
         <x:v>優先順位</x:v>
       </x:c>
     </x:row>
@@ -1359,18 +1353,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D10" s="34" t="str">
-        <x:v>完全取得</x:v>
-      </x:c>
-      <x:c r="E10" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F10" s="34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G10" s="34" t="str">
-        <x:v>部署構成、派遣社員有無、休憩環境を確認。</x:v>
-      </x:c>
-      <x:c r="H10" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E10" s="34" t="str">
+        <x:v>部署人数、男女比、派遣社員有無、年齢層、服装、施設を確認できているか。</x:v>
+      </x:c>
+      <x:c r="F10" s="17" t="str">
         <x:v>網羅性</x:v>
       </x:c>
     </x:row>
@@ -1385,18 +1373,12 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="D11" s="34" t="str">
-        <x:v>完全取得</x:v>
-      </x:c>
-      <x:c r="E11" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F11" s="34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G11" s="34" t="str">
-        <x:v>指揮命令者と合う人物像を確認。</x:v>
-      </x:c>
-      <x:c r="H11" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E11" s="34" t="str">
+        <x:v>指揮命令者の人柄、部署の雰囲気、合う人柄/避けたい人物像を確認できているか。</x:v>
+      </x:c>
+      <x:c r="F11" s="17" t="str">
         <x:v>網羅性/優先順位</x:v>
       </x:c>
     </x:row>
@@ -1411,18 +1393,12 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="D12" s="34" t="str">
-        <x:v>未取得</x:v>
-      </x:c>
-      <x:c r="E12" s="34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F12" s="34" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="G12" s="34" t="str">
-        <x:v>競合は確認。独占余地、決定者、決定日数が不足。</x:v>
-      </x:c>
-      <x:c r="H12" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E12" s="34" t="str">
+        <x:v>競合状況、独占期間、職場見学日時、決定者、決定までの日数を確認できているか。</x:v>
+      </x:c>
+      <x:c r="F12" s="17" t="str">
         <x:v>網羅性/クロージング</x:v>
       </x:c>
     </x:row>
@@ -1437,18 +1413,12 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="D13" s="34" t="str">
-        <x:v>未取得</x:v>
-      </x:c>
-      <x:c r="E13" s="34" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F13" s="34" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="G13" s="34" t="str">
-        <x:v>提案期限のみ。連絡方法と双方の次行動が未合意。</x:v>
-      </x:c>
-      <x:c r="H13" s="17" t="str">
+        <x:v>完全取得 / 部分取得 / 未取得</x:v>
+      </x:c>
+      <x:c r="E13" s="34" t="str">
+        <x:v>連絡方法、今後のスケジュール、具体的な次行動と期日を合意できているか。</x:v>
+      </x:c>
+      <x:c r="F13" s="17" t="str">
         <x:v>網羅性/クロージング</x:v>
       </x:c>
     </x:row>
@@ -1462,11 +1432,7 @@
       </x:c>
       <x:c r="D14" s="35" t="str"/>
       <x:c r="E14" s="35" t="str"/>
-      <x:c r="F14" s="35" t="n">
-        <x:v>36.5</x:v>
-      </x:c>
-      <x:c r="G14" s="35" t="str"/>
-      <x:c r="H14" s="19" t="str"/>
+      <x:c r="F14" s="19" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1478,7 +1444,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="26.3799991607666" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="95.08999633789062" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="97.55000305175781" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -1513,35 +1479,27 @@
         <x:v>改善インパクト = 重み × (1 - 取得率)。完全取得=1、部分取得=0.5、未取得=0。</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="24" hidden="0" customHeight="1">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="16" t="str">
         <x:v>選定</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
-        <x:v>改善インパクトが最大の項目を選ぶ。同点の場合は、クロージング/競合決定など商談成立に近い項目を優先、または表示順で後続重要項目を優先する。</x:v>
+        <x:v>改善インパクトが最大の項目を選ぶ。同点の場合は、商談成立に近い項目、または重みが高い項目を優先する。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
-        <x:v>今回最大</x:v>
+        <x:v>表示ルール</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
-        <x:v>連絡方法・スケジュール・ネクストステップ: 14 × (1 - 0) = 14。</x:v>
+        <x:v>項目名は12項目マスターの名称をそのまま表示する。短縮名やAIが作った別名は使わない。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="16" t="str">
-        <x:v>表示ルール</x:v>
-      </x:c>
-      <x:c r="B7" s="17" t="str">
-        <x:v>項目名は12項目マスターの名称をそのまま表示する。短縮名やAIが作った別名は使わない。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="18" t="str">
+      <x:c r="A7" s="18" t="str">
         <x:v>補足文</x:v>
       </x:c>
-      <x:c r="B8" s="19" t="str">
+      <x:c r="B7" s="19" t="str">
         <x:v>補足文や次回質問例はAIが生成してよい。ただし、元項目名とズレない表現にする。</x:v>
       </x:c>
     </x:row>
@@ -1556,10 +1514,9 @@
   <x:cols>
     <x:col min="1" max="1" width="6.75" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="20.25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="30.059999465942383" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="9.199999809265137" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="63.189998626708984" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="31.290000915527344" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="63.189998626708984" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="55.83000183105469" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="31.290000915527344" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -1570,15 +1527,12 @@
         <x:v>会話フロー項目</x:v>
       </x:c>
       <x:c r="C1" s="39" t="str">
-        <x:v>今回表示</x:v>
+        <x:v>判定の観点</x:v>
       </x:c>
       <x:c r="D1" s="39" t="str">
-        <x:v>判定</x:v>
-      </x:c>
-      <x:c r="E1" s="39" t="str">
-        <x:v>意味</x:v>
-      </x:c>
-      <x:c r="F1" s="27" t="str">
+        <x:v>表示例の考え方</x:v>
+      </x:c>
+      <x:c r="E1" s="27" t="str">
         <x:v>主に影響する大カテゴリ</x:v>
       </x:c>
     </x:row>
@@ -1590,15 +1544,12 @@
         <x:v>導入</x:v>
       </x:c>
       <x:c r="C2" s="34" t="str">
-        <x:v>論点提示あり</x:v>
+        <x:v>冒頭で目的・進め方・確認したい論点を置けているか。</x:v>
       </x:c>
       <x:c r="D2" s="34" t="str">
-        <x:v>実施</x:v>
-      </x:c>
-      <x:c r="E2" s="34" t="str">
-        <x:v>冒頭で本日の論点や進め方を置けている。</x:v>
-      </x:c>
-      <x:c r="F2" s="17" t="str">
+        <x:v>導入ができている場合は「論点提示あり」のように簡潔に表示する。</x:v>
+      </x:c>
+      <x:c r="E2" s="17" t="str">
         <x:v>商談の全体構成力/ヒアリングスキル</x:v>
       </x:c>
     </x:row>
@@ -1610,15 +1561,12 @@
         <x:v>背景</x:v>
       </x:c>
       <x:c r="C3" s="34" t="str">
-        <x:v>募集背景と不満点を確認</x:v>
+        <x:v>募集背景、現状課題、依頼理由を確認できているか。</x:v>
       </x:c>
       <x:c r="D3" s="34" t="str">
-        <x:v>実施</x:v>
-      </x:c>
-      <x:c r="E3" s="34" t="str">
-        <x:v>募集背景だけでなく、現行ベンダーへの不満まで確認できている。</x:v>
-      </x:c>
-      <x:c r="F3" s="17" t="str">
+        <x:v>背景の取得状況と、深掘りできた論点を短く表示する。</x:v>
+      </x:c>
+      <x:c r="E3" s="17" t="str">
         <x:v>網羅性/商談の全体構成力</x:v>
       </x:c>
     </x:row>
@@ -1630,15 +1578,12 @@
         <x:v>業務分解</x:v>
       </x:c>
       <x:c r="C4" s="34" t="str">
-        <x:v>主業務と条件を確認</x:v>
+        <x:v>職種名だけでなく、業務内容・1日の流れ・業務量に分解できているか。</x:v>
       </x:c>
       <x:c r="D4" s="34" t="str">
-        <x:v>実施</x:v>
-      </x:c>
-      <x:c r="E4" s="34" t="str">
-        <x:v>職種名で止まらず、業務内容や条件に分解できている。</x:v>
-      </x:c>
-      <x:c r="F4" s="17" t="str">
+        <x:v>主業務と条件の確認状況を表示する。</x:v>
+      </x:c>
+      <x:c r="E4" s="17" t="str">
         <x:v>網羅性/ヒアリングスキル</x:v>
       </x:c>
     </x:row>
@@ -1650,15 +1595,12 @@
         <x:v>優先順位</x:v>
       </x:c>
       <x:c r="C5" s="34" t="str">
-        <x:v>必須/歓迎/緩和可が浅い</x:v>
+        <x:v>必須条件・歓迎条件・緩和可能条件を分けられているか。</x:v>
       </x:c>
       <x:c r="D5" s="34" t="str">
-        <x:v>部分</x:v>
-      </x:c>
-      <x:c r="E5" s="34" t="str">
-        <x:v>条件の優先順位確認はあるが、候補者選定に使える粒度までは不足。</x:v>
-      </x:c>
-      <x:c r="F5" s="17" t="str">
+        <x:v>不足がある場合は、どの切り分けが浅いかを表示する。</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str">
         <x:v>優先順位の明確化</x:v>
       </x:c>
     </x:row>
@@ -1670,15 +1612,12 @@
         <x:v>職場環境</x:v>
       </x:c>
       <x:c r="C6" s="34" t="str">
-        <x:v>人物面まで確認</x:v>
+        <x:v>部署構成、雰囲気、合う人物像、NG人物像を確認できているか。</x:v>
       </x:c>
       <x:c r="D6" s="34" t="str">
-        <x:v>実施</x:v>
-      </x:c>
-      <x:c r="E6" s="34" t="str">
-        <x:v>職場環境や合う人物像まで確認できている。</x:v>
-      </x:c>
-      <x:c r="F6" s="17" t="str">
+        <x:v>人物面まで取れているかを表示する。</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str">
         <x:v>網羅性/優先順位の明確化</x:v>
       </x:c>
     </x:row>
@@ -1690,15 +1629,12 @@
         <x:v>競合・決定</x:v>
       </x:c>
       <x:c r="C7" s="34" t="str">
-        <x:v>決定者と日数が不足</x:v>
+        <x:v>競合状況、見学、決定者、決定までの日数を確認できているか。</x:v>
       </x:c>
       <x:c r="D7" s="34" t="str">
-        <x:v>不足</x:v>
-      </x:c>
-      <x:c r="E7" s="34" t="str">
-        <x:v>競合や見学後の決定プロセス・判断者・日数が不足している。</x:v>
-      </x:c>
-      <x:c r="F7" s="17" t="str">
+        <x:v>不足がある場合は、決定者・日数など具体的に表示する。</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str">
         <x:v>網羅性/クロージング</x:v>
       </x:c>
     </x:row>
@@ -1710,15 +1646,12 @@
         <x:v>要約・終話</x:v>
       </x:c>
       <x:c r="C8" s="35" t="str">
-        <x:v>期日合意はあるが連絡方法不足</x:v>
+        <x:v>要点、スケジュール、ネクストアクション、連絡方法を合意できているか。</x:v>
       </x:c>
       <x:c r="D8" s="35" t="str">
-        <x:v>部分</x:v>
-      </x:c>
-      <x:c r="E8" s="35" t="str">
-        <x:v>提案期限は合意できているが、連絡方法や双方の次行動が不足。</x:v>
-      </x:c>
-      <x:c r="F8" s="19" t="str">
+        <x:v>期日合意・連絡方法・双方の次行動の有無を表示する。</x:v>
+      </x:c>
+      <x:c r="E8" s="19" t="str">
         <x:v>クロージング/商談の全体構成力</x:v>
       </x:c>
     </x:row>
@@ -1733,7 +1666,7 @@
   <x:cols>
     <x:col min="1" max="1" width="27.610000610351562" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="54.599998474121094" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36.20000076293945" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="43.560001373291016" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -1744,7 +1677,7 @@
         <x:v>計算方法</x:v>
       </x:c>
       <x:c r="C1" s="27" t="str">
-        <x:v>今回例</x:v>
+        <x:v>補足</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
@@ -1755,7 +1688,7 @@
         <x:v>12項目の重み付き取得率 × 30点</x:v>
       </x:c>
       <x:c r="C2" s="17" t="str">
-        <x:v>0.74 × 30 = 22.2</x:v>
+        <x:v>12項目の判定をもとに算出する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -1763,10 +1696,10 @@
         <x:v>ヒアリングスキル</x:v>
       </x:c>
       <x:c r="B3" s="34" t="str">
-        <x:v>小カテゴリ平均を20点換算</x:v>
+        <x:v>小カテゴリ評価を20点換算</x:v>
       </x:c>
       <x:c r="C3" s="17" t="str">
-        <x:v>15.0</x:v>
+        <x:v>質問の仕方、深掘り、要約などを見る。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1774,10 +1707,10 @@
         <x:v>優先順位の明確化</x:v>
       </x:c>
       <x:c r="B4" s="34" t="str">
-        <x:v>小カテゴリ平均/加重を20点換算</x:v>
+        <x:v>小カテゴリ評価を20点換算</x:v>
       </x:c>
       <x:c r="C4" s="17" t="str">
-        <x:v>14.0</x:v>
+        <x:v>must/want/緩和可能条件の整理を見る。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -1788,7 +1721,7 @@
         <x:v>会話フロー達成度を10点換算</x:v>
       </x:c>
       <x:c r="C5" s="17" t="str">
-        <x:v>8.0</x:v>
+        <x:v>導入から終話までの流れを見る。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1799,7 +1732,7 @@
         <x:v>会話ログ上の振る舞い小カテゴリを10点換算</x:v>
       </x:c>
       <x:c r="C6" s="17" t="str">
-        <x:v>8.0</x:v>
+        <x:v>非言語要素は直接評価しない。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1810,7 +1743,7 @@
         <x:v>クロージング小カテゴリを10点換算</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
-        <x:v>7.0</x:v>
+        <x:v>期日と行動ベースの合意を見る。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1821,7 +1754,7 @@
         <x:v>6大カテゴリ点の合計</x:v>
       </x:c>
       <x:c r="C8" s="19" t="str">
-        <x:v>22.2 + 15.0 + 14.0 + 8.0 + 8.0 + 7.0 = 74.2</x:v>
+        <x:v>100点満点で表示する。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>